<commit_message>
Reclassifica R51 (FTFRUKI) de FALTA para PARCIAL: controle de mudanca evidenciado em GCO/GDE
</commit_message>
<xml_diff>
--- a/Checklist_MPS_SW_NivelC_FTFRUKI_PREENCHIDA.xlsx
+++ b/Checklist_MPS_SW_NivelC_FTFRUKI_PREENCHIDA.xlsx
@@ -2373,9 +2373,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>FALTA</t>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="E51" s="11" t="n"/>
@@ -2384,7 +2384,7 @@
       <c r="H51" s="11" t="n"/>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>Nenhum Change Request (TPL-GPR-006); TAE declara 'sem CR'; atraso/renomeacao tratados ad-hoc.</t>
+          <t>Controle de mudanca evidenciado em GCO §4 (CM-01..03, inclui ampliacao de escopo CM-03 aprovada) + GDE; sem formulario CR (TPL-GPR-006) e ha inconsistencia: TAE-002 §3 diz 'sem expansao de escopo' x GCO CM-03 'ampliacao de escopo'.</t>
         </is>
       </c>
     </row>

</xml_diff>